<commit_message>
Published state of ETDataset for deploy 2026-07
</commit_message>
<xml_diff>
--- a/nodes_source_analyses/energy/energy/energy_production_fischer_tropsch_biogenic_waste_ccs.xlsx
+++ b/nodes_source_analyses/energy/energy/energy_production_fischer_tropsch_biogenic_waste_ccs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10412"/>
   <workbookPr showInkAnnotation="0" codeName="ThisWorkbook" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mathijsbijkerk/Github/etdataset/nodes_source_analyses/energy/energy/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robin/Desktop/Quintel/etdataset/nodes_source_analyses/energy/energy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75CA544C-6847-4942-AC44-35D61B28FEBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1716BEE-7D41-E547-A931-09631201E407}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14460" yWindow="-33340" windowWidth="30080" windowHeight="16180" tabRatio="762" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1460" yWindow="500" windowWidth="28800" windowHeight="15820" tabRatio="762" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover sheet" sheetId="14" r:id="rId1"/>
@@ -42,7 +42,7 @@
     <definedName name="Wp_to_kWp">#REF!</definedName>
     <definedName name="WP_to_MWp">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr defaultImageDpi="32767"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="217">
   <si>
     <t>Source</t>
   </si>
@@ -830,6 +830,12 @@
   </si>
   <si>
     <t>Quintel</t>
+  </si>
+  <si>
+    <t>Is the actual CO2 capture rate</t>
+  </si>
+  <si>
+    <t>Taken from energy_hydrogen_biomass_gasification_ccs</t>
   </si>
 </sst>
 </file>
@@ -2377,7 +2383,6 @@
     <xf numFmtId="0" fontId="58" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="169" fontId="53" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="31" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="52" fillId="15" borderId="21" xfId="500" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="27" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2434,6 +2439,7 @@
     <xf numFmtId="0" fontId="55" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="53" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="501">
     <cellStyle name="Comma" xfId="496" builtinId="3"/>
@@ -3858,27 +3864,27 @@
       <c r="C4" s="19" t="s">
         <v>163</v>
       </c>
-      <c r="D4" s="180"/>
+      <c r="D4" s="179"/>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="1"/>
       <c r="B5" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="178" t="s">
+      <c r="C5" s="177" t="s">
         <v>157</v>
       </c>
-      <c r="D5" s="181"/>
+      <c r="D5" s="180"/>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="1"/>
       <c r="B6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="179" t="s">
+      <c r="C6" s="178" t="s">
         <v>214</v>
       </c>
-      <c r="D6" s="182"/>
+      <c r="D6" s="181"/>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="1"/>
@@ -3896,23 +3902,23 @@
         <v>24</v>
       </c>
       <c r="C9" s="45"/>
-      <c r="D9" s="180"/>
+      <c r="D9" s="179"/>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="1"/>
       <c r="B10" s="46"/>
-      <c r="C10" s="183"/>
-      <c r="D10" s="181"/>
+      <c r="C10" s="182"/>
+      <c r="D10" s="180"/>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="1"/>
       <c r="B11" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="184" t="s">
+      <c r="C11" s="183" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="181"/>
+      <c r="D11" s="180"/>
     </row>
     <row r="12" spans="1:4" ht="17" thickBot="1">
       <c r="A12" s="1"/>
@@ -3920,7 +3926,7 @@
       <c r="C12" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="181"/>
+      <c r="D12" s="180"/>
     </row>
     <row r="13" spans="1:4" ht="17" thickBot="1">
       <c r="A13" s="1"/>
@@ -3928,91 +3934,91 @@
       <c r="C13" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="181"/>
+      <c r="D13" s="180"/>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="1"/>
       <c r="B14" s="46"/>
-      <c r="C14" s="183" t="s">
+      <c r="C14" s="182" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="181"/>
+      <c r="D14" s="180"/>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="1"/>
       <c r="B15" s="46"/>
-      <c r="C15" s="183"/>
-      <c r="D15" s="181"/>
+      <c r="C15" s="182"/>
+      <c r="D15" s="180"/>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="1"/>
       <c r="B16" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="185" t="s">
+      <c r="C16" s="184" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="181"/>
+      <c r="D16" s="180"/>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="1"/>
       <c r="B17" s="46"/>
-      <c r="C17" s="186" t="s">
+      <c r="C17" s="185" t="s">
         <v>32</v>
       </c>
-      <c r="D17" s="181"/>
+      <c r="D17" s="180"/>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="1"/>
       <c r="B18" s="46"/>
-      <c r="C18" s="187" t="s">
+      <c r="C18" s="186" t="s">
         <v>33</v>
       </c>
-      <c r="D18" s="181"/>
+      <c r="D18" s="180"/>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="1"/>
       <c r="B19" s="46"/>
-      <c r="C19" s="188" t="s">
+      <c r="C19" s="187" t="s">
         <v>34</v>
       </c>
-      <c r="D19" s="181"/>
+      <c r="D19" s="180"/>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="1"/>
       <c r="B20" s="48"/>
-      <c r="C20" s="189" t="s">
+      <c r="C20" s="188" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="181"/>
+      <c r="D20" s="180"/>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="1"/>
       <c r="B21" s="48"/>
-      <c r="C21" s="190" t="s">
+      <c r="C21" s="189" t="s">
         <v>36</v>
       </c>
-      <c r="D21" s="181"/>
+      <c r="D21" s="180"/>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="1"/>
       <c r="B22" s="48"/>
-      <c r="C22" s="191" t="s">
+      <c r="C22" s="190" t="s">
         <v>37</v>
       </c>
-      <c r="D22" s="181"/>
+      <c r="D22" s="180"/>
     </row>
     <row r="23" spans="1:4">
       <c r="B23" s="48"/>
-      <c r="C23" s="192" t="s">
+      <c r="C23" s="191" t="s">
         <v>38</v>
       </c>
-      <c r="D23" s="181"/>
+      <c r="D23" s="180"/>
     </row>
     <row r="24" spans="1:4">
-      <c r="B24" s="193"/>
-      <c r="C24" s="194"/>
-      <c r="D24" s="182"/>
+      <c r="B24" s="192"/>
+      <c r="C24" s="193"/>
+      <c r="D24" s="181"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4040,30 +4046,30 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10">
-      <c r="B2" s="195" t="s">
+      <c r="B2" s="194" t="s">
         <v>64</v>
       </c>
-      <c r="C2" s="196"/>
-      <c r="D2" s="196"/>
-      <c r="E2" s="197"/>
+      <c r="C2" s="195"/>
+      <c r="D2" s="195"/>
+      <c r="E2" s="196"/>
     </row>
     <row r="3" spans="1:10">
-      <c r="B3" s="198"/>
-      <c r="C3" s="199"/>
-      <c r="D3" s="199"/>
-      <c r="E3" s="200"/>
+      <c r="B3" s="197"/>
+      <c r="C3" s="198"/>
+      <c r="D3" s="198"/>
+      <c r="E3" s="199"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="B4" s="198"/>
-      <c r="C4" s="199"/>
-      <c r="D4" s="199"/>
-      <c r="E4" s="200"/>
+      <c r="B4" s="197"/>
+      <c r="C4" s="198"/>
+      <c r="D4" s="198"/>
+      <c r="E4" s="199"/>
     </row>
     <row r="5" spans="1:10">
-      <c r="B5" s="201"/>
-      <c r="C5" s="202"/>
-      <c r="D5" s="202"/>
-      <c r="E5" s="203"/>
+      <c r="B5" s="200"/>
+      <c r="C5" s="201"/>
+      <c r="D5" s="201"/>
+      <c r="E5" s="202"/>
     </row>
     <row r="7" spans="1:10" ht="17" thickBot="1"/>
     <row r="8" spans="1:10">
@@ -4551,13 +4557,13 @@
       </c>
       <c r="E35" s="58">
         <f>Notes!D95</f>
-        <v>0.63278100000000004</v>
+        <v>0.9</v>
       </c>
       <c r="F35" s="54"/>
       <c r="G35" s="152"/>
       <c r="H35" s="54"/>
       <c r="I35" s="73" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="J35" s="57"/>
     </row>
@@ -4959,17 +4965,17 @@
       <c r="G7" s="41"/>
       <c r="K7" s="95"/>
       <c r="L7" s="96"/>
-      <c r="M7" s="204"/>
-      <c r="N7" s="205"/>
-      <c r="O7" s="205"/>
-      <c r="P7" s="205"/>
-      <c r="Q7" s="205"/>
-      <c r="R7" s="205"/>
-      <c r="S7" s="205"/>
-      <c r="T7" s="205"/>
-      <c r="U7" s="205"/>
-      <c r="V7" s="205"/>
-      <c r="W7" s="205"/>
+      <c r="M7" s="203"/>
+      <c r="N7" s="204"/>
+      <c r="O7" s="204"/>
+      <c r="P7" s="204"/>
+      <c r="Q7" s="204"/>
+      <c r="R7" s="204"/>
+      <c r="S7" s="204"/>
+      <c r="T7" s="204"/>
+      <c r="U7" s="204"/>
+      <c r="V7" s="204"/>
+      <c r="W7" s="204"/>
     </row>
     <row r="8" spans="1:23" ht="17" customHeight="1">
       <c r="A8" s="41"/>
@@ -6840,10 +6846,10 @@
       <c r="B70" s="85"/>
       <c r="C70" s="165"/>
       <c r="D70" s="163"/>
-      <c r="E70" s="206" t="s">
+      <c r="E70" s="205" t="s">
         <v>186</v>
       </c>
-      <c r="F70" s="206"/>
+      <c r="F70" s="205"/>
       <c r="G70" s="165"/>
       <c r="I70" s="165" t="s">
         <v>174</v>
@@ -7137,15 +7143,15 @@
       <c r="J81" s="165" t="s">
         <v>203</v>
       </c>
-      <c r="K81" s="177">
+      <c r="K81" s="176">
         <f>K80*K79</f>
         <v>1.2317052631578947E-2</v>
       </c>
-      <c r="L81" s="177">
+      <c r="L81" s="176">
         <f t="shared" ref="L81:M81" si="5">L80*L79</f>
         <v>7.4377263157894748E-3</v>
       </c>
-      <c r="M81" s="177">
+      <c r="M81" s="176">
         <f t="shared" si="5"/>
         <v>9.9361684210526324E-3</v>
       </c>
@@ -7401,15 +7407,14 @@
       <c r="C95" s="163" t="s">
         <v>182</v>
       </c>
-      <c r="D95" s="176">
-        <f>ROUND(G84/D81,6)</f>
-        <v>0.63278100000000004</v>
+      <c r="D95" s="147">
+        <v>0.9</v>
       </c>
       <c r="E95" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="F95" s="163" t="s">
-        <v>213</v>
+      <c r="F95" s="206" t="s">
+        <v>215</v>
       </c>
       <c r="G95" s="163"/>
       <c r="H95" s="163"/>

</xml_diff>